<commit_message>
feat: audit and integrate PathText (WsiCaption) dataset
- Implement src/audit_wsi_caption.py for streaming WSI tiles from NIH GDC
- Generate reports/preview_cpystan_wsi_caption.html with 8 diverse gigapixel slide overviews
- Update docs/datasets_histopatologia_multimodal.md with 9,009 audited cases across 30 TCGA projects
- Update docs/multimodal_datasets_matrix.xlsx with audited metrics and splits
- Synchronize comparative matrix in reports/index.html and reports/datasets_comparative_matrix.html
</commit_message>
<xml_diff>
--- a/docs/multimodal_datasets_matrix.xlsx
+++ b/docs/multimodal_datasets_matrix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,7 +541,6 @@
       <c r="I2" t="n">
         <v>6719</v>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>749.04 MB</t>
@@ -610,11 +609,9 @@
       <c r="G3" t="n">
         <v>985</v>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>985</v>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>505.50 MB</t>
@@ -683,9 +680,6 @@
       <c r="G4" t="n">
         <v>107000</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>855.79 MB</t>
@@ -760,7 +754,6 @@
       <c r="I5" t="n">
         <v>769</v>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>303.24 GB</t>
@@ -826,7 +819,6 @@
       <c r="F6" t="n">
         <v>10387</v>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>710</v>
       </c>
@@ -904,9 +896,6 @@
       <c r="G7" t="n">
         <v>223169</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>12.75 GB</t>
@@ -975,9 +964,6 @@
       <c r="G8" t="n">
         <v>186194</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>10.92 GB</t>
@@ -1046,9 +1032,6 @@
       <c r="G9" t="n">
         <v>1620876</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>933.28 MB</t>
@@ -1117,11 +1100,9 @@
       <c r="G10" t="n">
         <v>5000</v>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>2180</v>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>2.15 GB</t>
@@ -1153,6 +1134,293 @@
         </is>
       </c>
       <c r="Q10" t="inlineStr">
+        <is>
+          <t>Auditado</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>quilt-1m</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Quilt-1M</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>wisdomik/Quilt-1M</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Vision-Language Pretraining (VLP) &amp; Alignment</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Cross-Modal Retrieval, Zero-Shot Patch Classification</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1017712</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1004153</v>
+      </c>
+      <c r="H11" t="n">
+        <v>13559</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2.08 GB (CSV)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>~50+ GB (Imágenes)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>quilt_1m_lookup.csv + imágenes YouTube/PubMed/Twitter/OpenPath</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CC BY-NC-SA 4.0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Gated (Autenticado)</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>reports/preview_wisdomik_quilt_1m.html</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Auditado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>wsi-vqa</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>WSI-VQA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>cpystan/WSI-VQA</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Whole Slide Image Visual Question Answering</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Biomarker Prediction, Subtyping, Survival Prediction</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>8672</v>
+      </c>
+      <c r="G12" t="n">
+        <v>7139</v>
+      </c>
+      <c r="H12" t="n">
+        <v>798</v>
+      </c>
+      <c r="I12" t="n">
+        <v>735</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1.45 MB (JSON)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>~1 TB (WSIs en NIH GDC)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>WsiVQA_*.json + Láminas SVS en NIH GDC</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Abierto Directo</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>reports/preview_cpystan_wsi_vqa.html</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Auditado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>patchgastricadc22</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PatchGastricADC22</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Zenodo: 6021442</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Patch-Level Diagnostic Captioning &amp; Subtyping</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Histopathological Subtyping, Report Inference</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>262777</v>
+      </c>
+      <c r="G13" t="n">
+        <v>262777</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>7.20 GB (ZIP)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>7.20 GB (262,777 JPEG + CSV)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>patches_captions.zip + captions.csv (1,305 reportes)</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Zenodo / Open</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Abierto Directo</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>reports/preview_patch_gastric_adc22.html</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Auditado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>pathtext</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PathText (WsiCaption)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>cpystan/Wsi-Caption</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Whole Slide Image Captioning &amp; Report Generation</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>WSI Summarization, Molecular Subtyping via Report Extraction</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>9009</v>
+      </c>
+      <c r="G14" t="n">
+        <v>845</v>
+      </c>
+      <c r="H14" t="n">
+        <v>98</v>
+      </c>
+      <c r="I14" t="n">
+        <v>98</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>7.43 MB (JSON)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>~9 TB (WSIs en NIH GDC)</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>PathText.json + Láminas SVS en NIH GDC</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Abierto Directo</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>reports/preview_cpystan_wsi_caption.html</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>Auditado</t>
         </is>

</xml_diff>

<commit_message>
feat(datasets): audit ARCH dataset from local archives and generate preview report
- Implement src/audit_arch.py for non-destructive inspection of books_set.zip and pubmed_set.zip

- Track src/download_arch.py for multi-threaded downloading and integrity verification

- Generate reports/preview_arch.html with 13 representative visual-textual samples (multi-instance bags and singles)

- Audit 7,579 images and 7,614 captions across textbooks and PubMed articles (5.75 GB total)

- Document Warwick TIA sample disparity note and MIL bag structure in docs/datasets_histopatologia_multimodal.md

- Add ARCH to docs/multimodal_datasets_matrix.xlsx (row 15) and synchronize reports/index.html and datasets_comparative_matrix.html
</commit_message>
<xml_diff>
--- a/docs/multimodal_datasets_matrix.xlsx
+++ b/docs/multimodal_datasets_matrix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1421,6 +1421,71 @@
         </is>
       </c>
       <c r="Q14" t="inlineStr">
+        <is>
+          <t>Auditado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>arch</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ARCH (Multiple Instance Captioning)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Warwick TIA / CVPR 2021</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Multiple-Instance Captioning &amp; Dense Pathology Retrieval</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Multi-panel Subfigure Disambiguation, Representation Learning</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>7579</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>5.75 GB (ZIPs)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>~7.2 GB</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>ZIPs (PNG/JPG + captions.json)</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>CC BY-NC-SA 4.0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Abierto (TIA Warwick)</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>reports/preview_arch.html</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>Auditado</t>
         </is>

</xml_diff>